<commit_message>
Fix remaining shift mismatches in Sept 15.xlsx (Adrian Vernon, Reese Middleton on 9/17 & 9/20) to fully match locked roster
</commit_message>
<xml_diff>
--- a/2026-09-15/Sept 15.xlsx
+++ b/2026-09-15/Sept 15.xlsx
@@ -7195,7 +7195,7 @@
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>WO</t>
+          <t>07:00-15:30</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>WO</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="E180" s="6" t="inlineStr">
         <is>
-          <t>07:00-15:30</t>
+          <t>WO</t>
         </is>
       </c>
       <c r="F180" s="6" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="H180" s="6" t="inlineStr">
         <is>
-          <t>WO</t>
+          <t>07:00-15:30</t>
         </is>
       </c>
       <c r="I180" s="6" t="inlineStr">

</xml_diff>